<commit_message>
Move Pvt Ltd vs LLP vs OPC to today's test post; new topic for 30 Sep
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KtrHitBeTprcT6PzZjbJAv
</commit_message>
<xml_diff>
--- a/plan/content-plan-2026-09-27-to-2026-11-25.xlsx
+++ b/plan/content-plan-2026-09-27-to-2026-11-25.xlsx
@@ -712,12 +712,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Pvt Ltd vs LLP vs OPC – which should you choose?</t>
+          <t>Director vs shareholder – who does what in a Pvt Ltd?</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Liability, compliance load, funding, cost – side by side.</t>
+          <t>Roles, powers, liabilities and who signs which filings.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>